<commit_message>
Publish NBL27 and WNBL27 forecast and recommendation status
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -131,10 +131,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">GWS GIANTS</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gold Coast SUNS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GWS GIANTS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
Update model outputs 2026-09-13 21:29:57
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -131,10 +131,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">Gold Coast SUNS</t>
+  </si>
+  <si>
     <t xml:space="preserve">GWS GIANTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gold Coast SUNS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
Update model outputs 2026-09-15 20:33:09
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -131,10 +131,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">GWS GIANTS</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gold Coast SUNS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GWS GIANTS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
Update model outputs 2026-09-16 07:01:35
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t xml:space="preserve">Team</t>
   </si>
@@ -35,10 +35,10 @@
     <t xml:space="preserve">Sydney Swans</t>
   </si>
   <si>
-    <t xml:space="preserve">3.31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.89</t>
+    <t xml:space="preserve">3.54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.93</t>
   </si>
   <si>
     <t xml:space="preserve">1.00</t>
@@ -50,58 +50,46 @@
     <t xml:space="preserve">Fremantle</t>
   </si>
   <si>
-    <t xml:space="preserve">4.79</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.30</t>
+    <t xml:space="preserve">4.37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brisbane Lions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.68</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.35</t>
   </si>
   <si>
     <t xml:space="preserve">Hawthorn</t>
   </si>
   <si>
-    <t xml:space="preserve">6.85</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.26</t>
+    <t xml:space="preserve">6.23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.88</t>
   </si>
   <si>
     <t xml:space="preserve">Geelong Cats</t>
   </si>
   <si>
-    <t xml:space="preserve">7.54</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.78</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brisbane Lions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.65</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.70</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.81</t>
+    <t xml:space="preserve">16.81</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.31</t>
   </si>
   <si>
     <t xml:space="preserve">Adelaide Crows</t>
   </si>
   <si>
-    <t xml:space="preserve">18.08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.31</t>
+    <t xml:space="preserve">32.31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.80</t>
   </si>
   <si>
     <t xml:space="preserve">Melbourne</t>
@@ -110,16 +98,16 @@
     <t xml:space="preserve">60.06</t>
   </si>
   <si>
-    <t xml:space="preserve">23.81</t>
+    <t xml:space="preserve">23.31</t>
   </si>
   <si>
     <t xml:space="preserve">Western Bulldogs</t>
   </si>
   <si>
-    <t xml:space="preserve">120.48</t>
-  </si>
-  <si>
-    <t xml:space="preserve">50.25</t>
+    <t xml:space="preserve">129.03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">54.95</t>
   </si>
   <si>
     <t xml:space="preserve">Carlton</t>
@@ -557,7 +545,7 @@
         <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E4" t="s">
         <v>9</v>
@@ -568,16 +556,16 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>19</v>
       </c>
-      <c r="C5" t="s">
-        <v>20</v>
-      </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E5" t="s">
         <v>9</v>
@@ -588,16 +576,16 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" t="s">
         <v>22</v>
       </c>
-      <c r="B6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" t="s">
-        <v>24</v>
-      </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="E6" t="s">
         <v>9</v>
@@ -608,16 +596,16 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E7" t="s">
         <v>9</v>
@@ -628,13 +616,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -648,13 +636,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
         <v>10</v>
@@ -668,7 +656,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B10" t="s">
         <v>10</v>
@@ -688,7 +676,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B11" t="s">
         <v>10</v>
@@ -708,7 +696,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B12" t="s">
         <v>10</v>
@@ -728,7 +716,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B13" t="s">
         <v>10</v>
@@ -748,7 +736,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B14" t="s">
         <v>10</v>
@@ -768,7 +756,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B15" t="s">
         <v>10</v>
@@ -788,7 +776,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B16" t="s">
         <v>10</v>
@@ -808,7 +796,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B17" t="s">
         <v>10</v>
@@ -828,7 +816,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B18" t="s">
         <v>10</v>
@@ -848,7 +836,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B19" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Update model outputs 2026-09-17 05:21:14
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -119,10 +119,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">Gold Coast SUNS</t>
+  </si>
+  <si>
     <t xml:space="preserve">GWS GIANTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gold Coast SUNS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
Update model outputs 2026-09-19 21:35:03
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -119,10 +119,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">Gold Coast SUNS</t>
+  </si>
+  <si>
     <t xml:space="preserve">GWS GIANTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gold Coast SUNS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
Update model outputs 2026-09-24 12:13:31
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -35,10 +35,10 @@
     <t xml:space="preserve">Sydney Swans</t>
   </si>
   <si>
-    <t xml:space="preserve">3.54</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.93</t>
+    <t xml:space="preserve">3.70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.99</t>
   </si>
   <si>
     <t xml:space="preserve">1.00</t>
@@ -47,67 +47,67 @@
     <t xml:space="preserve">-</t>
   </si>
   <si>
+    <t xml:space="preserve">Brisbane Lions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.16</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fremantle</t>
   </si>
   <si>
-    <t xml:space="preserve">4.37</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brisbane Lions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.68</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.35</t>
+    <t xml:space="preserve">5.12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.41</t>
   </si>
   <si>
     <t xml:space="preserve">Hawthorn</t>
   </si>
   <si>
-    <t xml:space="preserve">6.23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.88</t>
+    <t xml:space="preserve">5.97</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.84</t>
   </si>
   <si>
     <t xml:space="preserve">Geelong Cats</t>
   </si>
   <si>
-    <t xml:space="preserve">16.81</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.31</t>
+    <t xml:space="preserve">16.45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.01</t>
   </si>
   <si>
     <t xml:space="preserve">Adelaide Crows</t>
   </si>
   <si>
-    <t xml:space="preserve">32.31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13.80</t>
+    <t xml:space="preserve">30.49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.88</t>
   </si>
   <si>
     <t xml:space="preserve">Melbourne</t>
   </si>
   <si>
-    <t xml:space="preserve">60.06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23.31</t>
+    <t xml:space="preserve">50.63</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23.20</t>
   </si>
   <si>
     <t xml:space="preserve">Western Bulldogs</t>
   </si>
   <si>
-    <t xml:space="preserve">129.03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">54.95</t>
+    <t xml:space="preserve">143.88</t>
+  </si>
+  <si>
+    <t xml:space="preserve">44.44</t>
   </si>
   <si>
     <t xml:space="preserve">Carlton</t>
@@ -119,10 +119,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">GWS GIANTS</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gold Coast SUNS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GWS GIANTS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
NBL projections 2026-09-26 08:23:54
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -119,10 +119,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">GWS GIANTS</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gold Coast SUNS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GWS GIANTS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
NBL projections 2026-10-02 20:22:46
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -119,10 +119,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">Gold Coast SUNS</t>
+  </si>
+  <si>
     <t xml:space="preserve">GWS GIANTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gold Coast SUNS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
Simplify model website navigation and projection views
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -119,10 +119,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">GWS GIANTS</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gold Coast SUNS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GWS GIANTS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
NBL projections 2026-10-05 10:22:40
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -119,10 +119,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">Gold Coast SUNS</t>
+  </si>
+  <si>
     <t xml:space="preserve">GWS GIANTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gold Coast SUNS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
Update model outputs 2026-10-05 17:46:16
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -119,10 +119,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">GWS GIANTS</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gold Coast SUNS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GWS GIANTS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
Update model outputs 2026-10-05 22:27:58
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -119,10 +119,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">Gold Coast SUNS</t>
+  </si>
+  <si>
     <t xml:space="preserve">GWS GIANTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gold Coast SUNS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
NBL and WNBL projections 2026-10-16 14:57:56
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -119,10 +119,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">GWS GIANTS</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gold Coast SUNS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GWS GIANTS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
Update model outputs 2026-10-16 22:27:00
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -119,10 +119,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">Gold Coast SUNS</t>
+  </si>
+  <si>
     <t xml:space="preserve">GWS GIANTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gold Coast SUNS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
Update model outputs 2026-10-18 11:45:13
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -119,10 +119,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">GWS GIANTS</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gold Coast SUNS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GWS GIANTS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
Update model outputs 2026-10-18 11:48:28
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -119,10 +119,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">Gold Coast SUNS</t>
+  </si>
+  <si>
     <t xml:space="preserve">GWS GIANTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gold Coast SUNS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
NBL and WNBL projections 2026-10-21 13:41:09
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -119,10 +119,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">GWS GIANTS</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gold Coast SUNS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GWS GIANTS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
NBL and WNBL projections 2026-10-21 15:28:24
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -119,10 +119,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">Gold Coast SUNS</t>
+  </si>
+  <si>
     <t xml:space="preserve">GWS GIANTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gold Coast SUNS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
NBL and WNBL projections 2026-10-22 10:44:14
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -119,10 +119,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">GWS GIANTS</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gold Coast SUNS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GWS GIANTS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
Update model outputs 2026-10-22 13:01:12
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -119,10 +119,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">Gold Coast SUNS</t>
+  </si>
+  <si>
     <t xml:space="preserve">GWS GIANTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gold Coast SUNS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
Refresh NBL WNBL A-League Men and Women 2026-10-27
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -119,10 +119,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">GWS GIANTS</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gold Coast SUNS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GWS GIANTS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>

<commit_message>
Update model outputs 2026-10-27 22:24:04
</commit_message>
<xml_diff>
--- a/files/AFL_futures_sim.xlsx
+++ b/files/AFL_futures_sim.xlsx
@@ -119,10 +119,10 @@
     <t xml:space="preserve">Essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">Gold Coast SUNS</t>
+  </si>
+  <si>
     <t xml:space="preserve">GWS GIANTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gold Coast SUNS</t>
   </si>
   <si>
     <t xml:space="preserve">North Melbourne</t>

</xml_diff>